<commit_message>
auto: 产出更新 2026-10-19 23:00
</commit_message>
<xml_diff>
--- a/霞浦发改批复_近半年.xlsx
+++ b/霞浦发改批复_近半年.xlsx
@@ -714,7 +714,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>申请中央预算内资金及地方财政配套</t>
+          <t>申请中央预算内资��及地方财政配套</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -2711,7 +2711,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>霞浦县县域医共体设备更新项目</t>
+          <t>霞浦县县域��共体设备更新项目</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">

</xml_diff>

<commit_message>
auto: 产出更新 2026-10-19 23:08
</commit_message>
<xml_diff>
--- a/霞浦发改批复_近半年.xlsx
+++ b/霞浦发改批复_近半年.xlsx
@@ -714,7 +714,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>申请中央预算内资��及地方财政配套</t>
+          <t>申请中央预算内资金及���方财政配套</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -2711,7 +2711,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>霞浦县县域��共体设备更新项目</t>
+          <t>霞浦县县域医共体设备更新项目</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">

</xml_diff>

<commit_message>
auto: 产出更新 2026-10-20 07:50
</commit_message>
<xml_diff>
--- a/霞浦发改批复_近半年.xlsx
+++ b/霞浦发改批复_近半年.xlsx
@@ -714,7 +714,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>申请中央预算内资金及���方财政配套</t>
+          <t>申请中央预算内资���及地方财政配��</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -2711,7 +2711,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>霞浦县县域医共体设备更新项目</t>
+          <t>霞浦县县域医共体设备更新��目</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">

</xml_diff>

<commit_message>
auto: 产出更新 2026-10-21 07:50
</commit_message>
<xml_diff>
--- a/霞浦发改批复_近半年.xlsx
+++ b/霞浦发改批复_近半年.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -524,219 +524,219 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>霞浦县东冲半岛北壁段旅游基础设施提升工程</t>
+          <t>“千鲜霞浦”文商旅综合体及大宗水产品交易中心项目配套路网建设工程</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>设计批复</t>
+          <t>可研批复</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕92号</t>
+          <t>霞发改审批〔2026〕96号</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>16713.94</v>
+        <v>35197.97</v>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>霞浦县北壁乡人民政府</t>
+          <t>霞浦县城市建设投资有限公司</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>霞浦县北壁乡</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr"/>
+          <t>福建省霞浦县松港组团</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>22个月</t>
+        </is>
+      </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>申请专项债资金及业主自筹</t>
+          <t>县财政配套</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260930_2487707.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202610/t20261016_2489809.htm</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>霞浦县沙江镇涵江村人居环境及生产道路提升项目</t>
+          <t>福建省霞浦县下洋城水库除险加固工程</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>设计批复</t>
+          <t>可研批复</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕91号</t>
+          <t>霞发改审批〔2026〕95号</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>142.23</v>
+        <v>306.02</v>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>霞浦县沙江镇人民政府</t>
+          <t>霞浦县长春镇人民政府</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>霞浦县沙江镇涵江村</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr"/>
+          <t>霞浦县长春镇下洋城村</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>8个月</t>
+        </is>
+      </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>申请中央专项彩票公益金及业主自筹</t>
+          <t>申请中央财政资金补助及县财政配套</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260930_2487705.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202610/t20261016_2489805.htm</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>霞浦县盐田畲族乡水升海堤除险修复工程</t>
+          <t>霞浦县东冲半岛北壁段旅游基础设施提升工程</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>可研批复</t>
+          <t>设计批复</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕90号</t>
+          <t>霞发改审批〔2026〕92号</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>270.75</v>
+        <v>16713.94</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>霞浦县盐田畲族乡人民政府</t>
+          <t>霞浦县北壁乡人民政府</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>霞浦县盐田畲族乡水升村</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>6个月</t>
-        </is>
-      </c>
+          <t>霞浦县北壁乡</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>申请中央预算内资金及地方财政配套</t>
+          <t>申请专项债资金及业主自筹</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482424.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260930_2487707.htm</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>松城街道水毁道路灾后修复项目</t>
+          <t>霞浦县沙江镇涵江村人居环境及生产道路提升项目</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>可研批复</t>
+          <t>设计批复</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕89号</t>
+          <t>霞发改审批〔2026〕91号</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>297.0299</v>
+        <v>142.23</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>霞浦县人民政府松城街道办事处</t>
+          <t>霞浦县沙江镇人民政府</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>霞浦县松城街道</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>3个月</t>
-        </is>
-      </c>
+          <t>霞浦县沙江镇涵江村</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>申请中央预算内资���及地方财政配��</t>
+          <t>申请中央专项彩票公益金及业主自筹</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482423.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260930_2487705.htm</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>霞浦县松港街道竹下村罗汉溪引水渠道修复工程</t>
+          <t>霞浦县盐田畲族乡水升海堤除险修复工程</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -746,20 +746,20 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕88号</t>
+          <t>霞发改审批〔2026〕90号</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>218.23</v>
+        <v>270.75</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>霞浦县人民政府松港街道办事处</t>
+          <t>霞浦县盐田畲族乡人民政府</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>霞浦县松港街道竹下村</t>
+          <t>霞浦县盐田畲族乡水升村</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -784,14 +784,14 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482422.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482424.htm</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>霞浦县牙城镇灾毁修复项目</t>
+          <t>松城街道水毁道路灾后修复项目</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -801,25 +801,25 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕87号</t>
+          <t>霞发改审批〔2026〕89号</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>243.37</v>
+        <v>297.0299</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>霞浦县牙城镇人民政府</t>
+          <t>霞浦县人民政府松城街道办事处</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>霞浦县牙城镇</t>
+          <t>霞浦县松城街道</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>10个月</t>
+          <t>3个月</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -839,14 +839,14 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482416.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482423.htm</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>霞浦县水门畲族乡道路水毁塌方修复工程</t>
+          <t>霞浦县松港街道竹下村罗汉溪引水渠道修复工程</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -856,25 +856,25 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕86号</t>
+          <t>霞发改审批〔2026〕88号</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>252.3706</v>
+        <v>218.23</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>霞浦县水门畲族乡人民政府</t>
+          <t>霞浦县人民政府松港街道办事处</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>霞浦县水门畲族乡</t>
+          <t>霞浦县松港街道竹下村</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>3个月</t>
+          <t>6个月</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
@@ -894,48 +894,52 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482415.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482422.htm</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>“千鲜霞浦”文商旅综合体及大宗水产品交易中心项目配套路网建设工程建议书</t>
+          <t>霞浦县牙城镇灾毁修复项目</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>立项批复</t>
+          <t>可研批复</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕85号</t>
+          <t>霞发改审批〔2026〕87号</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>38232.61</v>
+        <v>243.37</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>霞浦县城市建设投资有限公司</t>
+          <t>霞浦县牙城镇人民政府</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>福建省霞浦县松港组团</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr"/>
+          <t>霞浦县牙城镇</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>10个月</t>
+        </is>
+      </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>县财政资金</t>
+          <t>申请中央预算内资金及地方财政配套</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -945,48 +949,52 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482414.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482416.htm</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>霞浦县松城街道青福村道路沿线设施提升及人居环境改造项目</t>
+          <t>霞浦县水门畲族乡道路水毁塌方修复工程</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>设计批复</t>
+          <t>可研批复</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕83号</t>
+          <t>霞发改审批〔2026〕86号</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>173.45</v>
+        <v>252.3706</v>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>霞浦县人民政府松城街道办事处</t>
+          <t>霞浦县水门畲族乡人民政府</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>霞浦县松城街道青福村</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr"/>
+          <t>霞浦县水门畲族乡</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>3个月</t>
+        </is>
+      </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>申请中央专项彩票公益金及业主自筹</t>
+          <t>申请中央预算内资金及地方财政配套</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
@@ -996,48 +1004,48 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482410.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482415.htm</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>霞浦县松港街道八斗浿村道路沿线设施及休闲文化广场改造提升项目</t>
+          <t>“千鲜霞浦”文商旅综合体及大宗水产品交易中心项目配套路网建设工程建议书</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>设计批复</t>
+          <t>立项批复</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕82号</t>
+          <t>霞发改审批〔2026〕85号</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>130.23</v>
+        <v>38232.61</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>霞浦县人民政府松港街道办事处</t>
+          <t>霞浦县城市建设投资有限公司</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>霞浦县松港街道八斗浿村</t>
+          <t>福建省霞浦县松港组团</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr"/>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>申请中央专项彩票公益金及业主自筹</t>
+          <t>县财政资金</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
@@ -1047,48 +1055,48 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482409.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482414.htm</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>霞浦县县域医共体资源共享能力提升</t>
+          <t>霞浦县松城街道青福村道路沿线设施提升及人居环境改造项目</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>立项批复</t>
+          <t>设计批复</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕81号</t>
+          <t>霞发改审批〔2026〕83号</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>8500</v>
+        <v>173.45</v>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>霞浦县总医院</t>
+          <t>霞浦县人民政府松城街道办事处</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>霞浦县医院、霞浦县中医院新院区</t>
+          <t>霞浦县松城街道青福村</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr"/>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>争取中央及省级医疗卫生领域补助资金、县财政统筹安排及项目单位多渠道自筹</t>
+          <t>申请中央专项彩票公益金及业主自筹</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
@@ -1098,69 +1106,65 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482407.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482410.htm</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>霞浦县入河排污口整治及规范化建设工程</t>
+          <t>霞浦县松港街道八斗浿村道路沿线设施及休闲文化广场改造提升项目</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>可研批复</t>
+          <t>设计批复</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕80号</t>
+          <t>霞发改审批〔2026〕82号</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>6480.87</v>
+        <v>130.23</v>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>霞浦县水利投资有限公司</t>
+          <t>霞浦县人民政府松港街道办事处</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>霞浦县松城街道，以三河流域上游玉潭溪、石贝溪及三河干流等重要水体为治理重点，范围</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>24个月</t>
-        </is>
-      </c>
+          <t>霞浦县松港街道八斗浿村</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>中央水污染防治资金和地方财政资金</t>
+          <t>申请中央专项彩票公益金及业主自筹</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260901_2479038.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482409.htm</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>霞浦县入河排污口整治及规范化建设工程建议书</t>
+          <t>霞浦县县域医共体资源共享能力提升</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1170,48 +1174,48 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕78号</t>
+          <t>霞发改审批〔2026〕81号</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>6480.87</v>
+        <v>8500</v>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>霞浦县水利投资有限公司</t>
+          <t>霞浦县总医院</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>霞浦县松城街道</t>
+          <t>霞浦县医院、霞浦县中医院新院区</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr"/>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>中央预算内资金和地方财政配套</t>
+          <t>争取中央及省级医疗卫生领域补助资金、县财政统筹安排及项目单位多渠道自筹</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260901_2479034.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482407.htm</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>霞浦县柏洋乡饮用水源保护区环境综合整治与生态修复项目</t>
+          <t>霞浦县入河排污口整治及规范化建设工程</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1221,35 +1225,35 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕77号</t>
+          <t>霞发改审批〔2026〕80号</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>511.06</v>
+        <v>6480.87</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>霞浦县柏洋乡人民政府</t>
+          <t>霞浦县水利投资有限公司</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>福建省宁德市霞浦县柏洋乡</t>
+          <t>霞浦县松城街道，以三河流域上游玉潭溪、石贝溪及三河干流等重要水体为治理重点，范围</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>12个月</t>
+          <t>24个月</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>县级饮用水源地生态补偿项目资金</t>
+          <t>中央水污染防治资金和地方财政资金</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
@@ -1259,150 +1263,154 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260901_2479031.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260901_2479038.htm</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>溪南镇南岸村基础设施提升改造项目</t>
+          <t>霞浦县入河排污口整治及规范化建设工程建议书</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>设计批复</t>
+          <t>立项批复</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕74号</t>
+          <t>霞发改审批〔2026〕78号</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>153.36</v>
+        <v>6480.87</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>霞浦县溪南镇人民政府</t>
+          <t>霞浦县水利投资有限公司</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>霞浦县溪南镇南岸村</t>
+          <t>霞浦县松城街道</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr"/>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>申请中央专项彩票公益金及业主自筹</t>
+          <t>中央预算内资金和地方财政配套</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202608/t20260803_2473774.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260901_2479034.htm</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>霞浦县城区排水设施提升改造工程（一期）C标段</t>
+          <t>霞浦县柏洋乡饮用水源保护区环境综合整治与生态修复项目</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>设计批复</t>
+          <t>可研批复</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕70号</t>
+          <t>霞发改审批〔2026〕77号</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>17379.04</v>
+        <v>511.06</v>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>霞浦县城市建设投资有限公司</t>
+          <t>霞浦县柏洋乡人民政府</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>霞浦县城区</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr"/>
+          <t>福建省宁德市霞浦县柏洋乡</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>12个月</t>
+        </is>
+      </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>申请超长期特别国家债券及财政局统筹安排</t>
+          <t>县级饮用水源地生态补偿项目资金</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202608/t20260803_2473762.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260901_2479031.htm</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>霞浦县第八中学松兴校区篮球场建设工程</t>
+          <t>溪南镇南岸村基础设施提升改造项目</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>立项批复</t>
+          <t>设计批复</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕69号</t>
+          <t>霞发改审批〔2026〕74号</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>112.08</v>
+        <v>153.36</v>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>霞浦县第八中学</t>
+          <t>霞浦县溪南镇人民政府</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>霞浦县松城街道松兴社区曲井巷33号</t>
+          <t>霞浦县溪南镇南岸村</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr"/>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>县财政统筹安排</t>
+          <t>申请中央专项彩票公益金及业主自筹</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
@@ -1412,120 +1420,116 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202608/t20260803_2473758.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202608/t20260803_2473774.htm</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>霞浦县水门片区冷链物流项目</t>
+          <t>霞浦县城区排水设施提升改造工程（一期）C标段</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>可研批复</t>
+          <t>设计批复</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕68号</t>
+          <t>霞发改审批〔2026〕70号</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11836.82</v>
+        <v>17379.04</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>福建鑫水门投资发展有限公司</t>
+          <t>霞浦县城市建设投资有限公司</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>霞浦县水门畲族乡</t>
+          <t>霞浦县城区</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr"/>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>申请专项债资金及由县、乡镇财政统筹</t>
+          <t>申请超长期特别国家债券及财政局统筹安排</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202607/t20260717_2471081.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202608/t20260803_2473762.htm</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>霞浦东冲半岛外海道路工程-石人下段</t>
+          <t>霞浦县第八中学松兴校区篮球场建设工程</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>可研批复</t>
+          <t>立项批复</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕65号</t>
+          <t>霞发改审批〔2026〕69号</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1915.8585</v>
+        <v>112.08</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>霞浦县旅游投资发展有限公司</t>
+          <t>霞浦县第八中学</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>霞浦县北壁乡</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>3个月</t>
-        </is>
-      </c>
+          <t>霞浦县松城街道松兴社区曲井巷33号</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>县财政拨款</t>
+          <t>县财政统筹安排</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202607/t20260717_2471075.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202608/t20260803_2473758.htm</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>霞浦县公立医院能力提升项目</t>
+          <t>霞浦县水门片区冷链物流项目</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1535,52 +1539,48 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕64号</t>
+          <t>霞发改审批〔2026〕68号</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>9082.120000000001</v>
+        <v>11836.82</v>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>霞浦县总医院</t>
+          <t>福建鑫水门投资发展有限公司</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>霞浦县医院、县中医院、各乡镇卫生院</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>24个月</t>
-        </is>
-      </c>
+          <t>霞浦县水门畲族乡</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr"/>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>申请中央预算内补助及财政统筹</t>
+          <t>申请专项债资金及由县、乡镇财政统筹</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202607/t20260701_2467446.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202607/t20260717_2471081.htm</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>霞浦县三沙镇区基础配套设施改造提升项目</t>
+          <t>霞浦东冲半岛外海道路工程-石人下段</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1590,52 +1590,52 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕63号</t>
+          <t>霞发改审批〔2026〕65号</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>589.9299999999999</v>
+        <v>1915.8585</v>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>霞浦县三沙镇人民政府</t>
+          <t>霞浦县旅游投资发展有限公司</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>霞浦县三沙镇</t>
+          <t>霞浦县北壁乡</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>6个月</t>
+          <t>3个月</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>申请公益性基金及业主自筹</t>
+          <t>县财政拨款</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202607/t20260701_2467439.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202607/t20260717_2471075.htm</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>霞浦经济开发区渔洋里片区污水处理厂项目</t>
+          <t>霞浦县公立医院能力提升项目</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1645,31 +1645,35 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕62号</t>
+          <t>霞发改审批〔2026〕64号</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>6774</v>
+        <v>9082.120000000001</v>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>福建省霞浦经济开发区投资建设有限公司</t>
+          <t>霞浦县总医院</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>霞浦县渔洋里片区</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr"/>
+          <t>霞浦县医院、县中医院、各乡镇卫生院</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>24个月</t>
+        </is>
+      </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>县财政配套及建设单位自筹</t>
+          <t>申请中央预算内补助及财政统筹</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
@@ -1679,14 +1683,14 @@
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202607/t20260701_2467437.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202607/t20260701_2467446.htm</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>溪南镇南岸村基础设施提升改造项目</t>
+          <t>霞浦县三沙镇区基础配套设施改造提升项目</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1696,35 +1700,35 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕60号</t>
+          <t>霞发改审批〔2026〕63号</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>156.82</v>
+        <v>589.9299999999999</v>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>霞浦县溪南镇人民政府</t>
+          <t>霞浦县三沙镇人民政府</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>霞浦县溪南镇南岸村</t>
+          <t>霞浦县三沙镇</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>8个月</t>
+          <t>6个月</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>申请中央专项彩票公益金及业主自筹</t>
+          <t>申请公益性基金及业主自筹</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
@@ -1734,14 +1738,14 @@
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202607/t20260701_2467431.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202607/t20260701_2467439.htm</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>霞浦县城乡公交基础设施全域提升工程</t>
+          <t>霞浦经济开发区渔洋里片区污水处理厂项目</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1751,35 +1755,31 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕59号</t>
+          <t>霞发改审批〔2026〕62号</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>15804.49</v>
+        <v>6774</v>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>霞浦县交通运输事业发展中心</t>
+          <t>福建省霞浦经济开发区投资建设有限公司</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>霞浦县</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>24个月</t>
-        </is>
-      </c>
+          <t>霞浦县渔洋里片区</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr"/>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>申请专项债资金及财政筹集配套</t>
+          <t>县财政配套及建设单位自筹</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
@@ -1789,65 +1789,69 @@
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202607/t20260701_2467422.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202607/t20260701_2467437.htm</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>霞浦县北壁乡2025年公益性基础设施建设项目</t>
+          <t>溪南镇南岸村基础设施提升改造项目</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>设计批复</t>
+          <t>可研批复</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕58号</t>
+          <t>霞发改审批〔2026〕60号</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>447.01</v>
+        <v>156.82</v>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>霞浦县北壁乡人民政府</t>
+          <t>霞浦县溪南镇人民政府</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>霞浦县北壁乡</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr"/>
+          <t>霞浦县溪南镇南岸村</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>8个月</t>
+        </is>
+      </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>中央专项资金补助及业主自筹</t>
+          <t>申请中央专项彩票公益金及业主自筹</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202606/t20260615_2464208.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202607/t20260701_2467431.htm</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>霞浦东冲半岛外海道路工程 （外浒1号桥段）</t>
+          <t>霞浦县城乡公交基础设施全域提升工程</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1857,90 +1861,86 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕57号</t>
+          <t>霞发改审批〔2026〕59号</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>2142.6612</v>
+        <v>15804.49</v>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>霞浦县旅游投资发展有限公司</t>
+          <t>霞浦县交通运输事业发展中心</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>霞浦县下浒镇</t>
+          <t>霞浦县</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>18个月</t>
+          <t>24个月</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>财政拨款</t>
+          <t>申请专项债资金及财政筹集配套</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202606/t20260615_2464207.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202607/t20260701_2467422.htm</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>霞浦东冲半岛外海道路工程 （北兜至视界园段）</t>
+          <t>霞浦县北壁乡2025年公益性基础设施建设项目</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>可研批复</t>
+          <t>设计批复</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕56号</t>
+          <t>霞发改审批〔2026〕58号</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>12497.8421</v>
+        <v>447.01</v>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>霞浦县旅游投资发展有限公司</t>
+          <t>霞浦县北壁乡人民政府</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>霞浦县松山街道、长春镇</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>18个月</t>
-        </is>
-      </c>
+          <t>霞浦县北壁乡</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>县财政拨款</t>
+          <t>中央专项资金补助及业主自筹</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
@@ -1950,185 +1950,209 @@
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202606/t20260615_2464198.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202606/t20260615_2464208.htm</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>霞浦经济开发区渔洋里片区基础设施配套提升工程建议书</t>
+          <t>霞浦东冲半岛外海道路工程 （外浒1号桥段）</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>立项批复</t>
+          <t>可研批复</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕54号</t>
+          <t>霞发改审批〔2026〕57号</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>1137.68</v>
+        <v>2142.6612</v>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>福建省霞浦经济开发区投资建设有限公司</t>
+          <t>霞浦县旅游投资发展有限公司</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>霞浦县经济开发区</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr"/>
+          <t>霞浦县下浒镇</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>18个月</t>
+        </is>
+      </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>霞浦县地方政府财政资金</t>
+          <t>财政拨款</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202606/t20260601_2461061.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202606/t20260615_2464207.htm</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>霞浦县综合高中建设</t>
+          <t>霞浦东冲半岛外海道路工程 （北兜至视界园段）</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>立项批复</t>
+          <t>可研批复</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕53号</t>
+          <t>霞发改审批〔2026〕56号</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>79480.03</v>
+        <v>12497.8421</v>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>霞浦县教育局</t>
+          <t>霞浦县旅游投资发展有限公司</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>霞浦县松港街道</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr"/>
+          <t>霞浦县松山街道、长春镇</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>18个月</t>
+        </is>
+      </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>申请地方政府专项债、中央预算资金及财政配套资金</t>
+          <t>县财政拨款</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459220.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202606/t20260615_2464198.htm</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>霞浦县乡镇污水处理提升改造工程二期—（沙江镇）</t>
+          <t>霞浦经济开发区渔洋里片区基础设施配套提升工程建议书</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>设计批复</t>
+          <t>立项批复</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕52号</t>
+          <t>霞发改审批〔2026〕54号</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>1714.21</v>
+        <v>1137.68</v>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>霞浦县沙江镇人民政府</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr"/>
+          <t>福建省霞浦经济开发区投资建设有限公司</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>霞浦县经济开发区</t>
+        </is>
+      </c>
       <c r="G31" s="3" t="inlineStr"/>
-      <c r="H31" s="3" t="inlineStr"/>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>霞浦县地方政府财政资金</t>
+        </is>
+      </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459219.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202606/t20260601_2461061.htm</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>霞浦县乡镇污水处理提升改造工程二期（长春镇）</t>
+          <t>霞浦县综合高中建设</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>设计批复</t>
+          <t>立项批复</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕51号</t>
+          <t>霞发改审批〔2026〕53号</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>1105.17</v>
+        <v>79480.03</v>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>霞浦县长春镇人民政府</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr"/>
+          <t>霞浦县教育局</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>霞浦县松港街道</t>
+        </is>
+      </c>
       <c r="G32" s="3" t="inlineStr"/>
-      <c r="H32" s="3" t="inlineStr"/>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>申请地方政府专项债、中央预算资金及财政配套资金</t>
+        </is>
+      </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
@@ -2138,45 +2162,37 @@
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459218.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459220.htm</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>霞浦县第七小学学生宿舍楼及食堂建设</t>
+          <t>霞浦县乡镇污水处理提升改造工程二期—（沙江镇）</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>立项批复</t>
+          <t>设计批复</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕50号</t>
+          <t>霞发改审批〔2026〕52号</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>3886.23</v>
+        <v>1714.21</v>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>霞浦县第七小学</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>霞浦县第七小学校内</t>
-        </is>
-      </c>
+          <t>霞浦县沙江镇人民政府</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr"/>
       <c r="G33" s="3" t="inlineStr"/>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>县财政教育专项经费中统筹安排</t>
-        </is>
-      </c>
+      <c r="H33" s="3" t="inlineStr"/>
       <c r="I33" s="3" t="inlineStr">
         <is>
           <t>2026-05-15</t>
@@ -2189,14 +2205,14 @@
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459215.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459219.htm</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>霞浦县乡镇污水处理提升改造工程（二期）-溪南镇</t>
+          <t>霞浦县乡镇污水处理提升改造工程二期（长春镇）</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -2206,15 +2222,15 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕49号</t>
+          <t>霞发改审批〔2026〕51号</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>3728.96</v>
+        <v>1105.17</v>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>霞浦县溪南镇人民政府</t>
+          <t>霞浦县长春镇人民政府</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr"/>
@@ -2222,7 +2238,7 @@
       <c r="H34" s="3" t="inlineStr"/>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
@@ -2232,52 +2248,48 @@
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459214.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459218.htm</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>霞浦下浒全民健身中心项目</t>
+          <t>霞浦县第七小学学生宿舍楼及食堂建设</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>可研批复</t>
+          <t>立项批复</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕47号</t>
+          <t>霞发改审批〔2026〕50号</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>3793.46</v>
+        <v>3886.23</v>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>霞浦县下浒镇人民政府</t>
+          <t>霞浦县第七小学</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>霞浦县下浒镇</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>24个月</t>
-        </is>
-      </c>
+          <t>霞浦县第七小学校内</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr"/>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>申请专项债资金及县、乡镇财政统筹</t>
+          <t>县财政教育专项经费中统筹安排</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
@@ -2287,14 +2299,14 @@
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459211.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459215.htm</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>霞浦县乡镇污水提升改造工程二期（盐田畲族乡）</t>
+          <t>霞浦县乡镇污水处理提升改造工程（二期）-溪南镇</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -2304,15 +2316,15 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕46号</t>
+          <t>霞发改审批〔2026〕49号</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>345.5</v>
+        <v>3728.96</v>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>霞浦县盐田畲族乡人民政府</t>
+          <t>霞浦县溪南镇人民政府</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr"/>
@@ -2320,7 +2332,7 @@
       <c r="H36" s="3" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
@@ -2330,40 +2342,52 @@
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459210.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459214.htm</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>霞浦县乡镇污水处理提升改造工程二期-(北壁乡)</t>
+          <t>霞浦下浒全民健身中心项目</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>设计批复</t>
+          <t>可研批复</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕45号</t>
+          <t>霞发改审批〔2026〕47号</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>2430.38</v>
+        <v>3793.46</v>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>霞浦县北壁乡人民政府</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr"/>
-      <c r="G37" s="3" t="inlineStr"/>
-      <c r="H37" s="3" t="inlineStr"/>
+          <t>霞浦县下浒镇人民政府</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>霞浦县下浒镇</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>24个月</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>申请专项债资金及县、乡镇财政统筹</t>
+        </is>
+      </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
@@ -2373,14 +2397,14 @@
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459209.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459211.htm</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>霞浦县黄瓜山路（松山大道-六一七路）道路工程</t>
+          <t>霞浦县乡镇污水提升改造工程二期（盐田畲族乡）</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -2390,48 +2414,40 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕44号</t>
+          <t>霞发改审批〔2026〕46号</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>2551.24</v>
+        <v>345.5</v>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>霞浦县城市建设投资有限公司</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>霞浦县松港组团</t>
-        </is>
-      </c>
+          <t>霞浦县盐田畲族乡人民政府</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr"/>
       <c r="G38" s="3" t="inlineStr"/>
-      <c r="H38" s="3" t="inlineStr">
-        <is>
-          <t>财政拨款</t>
-        </is>
-      </c>
+      <c r="H38" s="3" t="inlineStr"/>
       <c r="I38" s="3" t="inlineStr">
         <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="J38" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459208.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459210.htm</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>霞浦县乡镇污水处理提升改造工程(二期)-下浒镇上澳村等9个村农村污水治理项目</t>
+          <t>霞浦县乡镇污水处理提升改造工程二期-(北壁乡)</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -2441,15 +2457,15 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕43号</t>
+          <t>霞发改审批〔2026〕45号</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>1793.37</v>
+        <v>2430.38</v>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>霞浦县下浒镇人民政府</t>
+          <t>霞浦县北壁乡人民政府</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr"/>
@@ -2457,7 +2473,7 @@
       <c r="H39" s="3" t="inlineStr"/>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
@@ -2467,65 +2483,65 @@
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459207.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459209.htm</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>福建省霞浦县海洋牧场深水抗风浪网箱养殖项目</t>
+          <t>霞浦县黄瓜山路（松山大道-六一七路）道路工程</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>可研批复</t>
+          <t>设计批复</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕39号</t>
+          <t>霞发改审批〔2026〕44号</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>24014</v>
+        <v>2551.24</v>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>福建省霞浦县光大渔港开发有限公司</t>
+          <t>霞浦县城市建设投资有限公司</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>霞浦县长春镇加竹村长草屿附近海域</t>
+          <t>霞浦县松港组团</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr"/>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>申请专项债资金及财政资金</t>
+          <t>财政拨款</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202604/t20260430_2455988.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459208.htm</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>霞浦县松城街道西南片区老旧小区改造（四期）</t>
+          <t>霞浦县乡镇污水处理提升改造工程(二期)-下浒镇上澳村等9个村农村污水治理项目</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -2535,41 +2551,33 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕40号</t>
+          <t>霞发改审批〔2026〕43号</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>5843.66</v>
+        <v>1793.37</v>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>霞浦县人民政府松城街道办事处</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>霞浦县松城街道</t>
-        </is>
-      </c>
+          <t>霞浦县下浒镇人民政府</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr"/>
       <c r="G41" s="3" t="inlineStr"/>
-      <c r="H41" s="3" t="inlineStr">
-        <is>
-          <t>申请专项债资金</t>
-        </is>
-      </c>
+      <c r="H41" s="3" t="inlineStr"/>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202604/t20260430_2455983.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459207.htm</t>
         </is>
       </c>
     </row>
@@ -2581,16 +2589,16 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>设计批复</t>
+          <t>可研批复</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕41号</t>
+          <t>霞发改审批〔2026〕39号</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>23938.04</v>
+        <v>24014</v>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
@@ -2619,6 +2627,108 @@
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202604/t20260430_2455988.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>霞浦县松城街道西南片区老旧小区改造（四期）</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>设计批复</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>霞发改审批〔2026〕40号</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>5843.66</v>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>霞浦县人民政府松城街道办事处</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>霞浦县松城街道</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr"/>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>申请专项债资金</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202604/t20260430_2455983.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>福建省霞浦县海洋牧场深水抗风浪网箱养殖项目</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>设计批复</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>霞发改审批〔2026〕41号</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>23938.04</v>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>福建省霞浦县光大渔港开发有限公司</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>霞浦县长春镇加竹村长草屿附近海域</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr"/>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>申请专项债资金及财政资金</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
         <is>
           <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202604/t20260430_2455979.htm</t>
         </is>
@@ -2635,7 +2745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2711,109 +2821,89 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>霞浦县县域医共体设备更新��目</t>
+          <t>同意文武水闸除险加固项目法人</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>可研批复</t>
+          <t>变更撤销类</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕84号</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>2789.32</v>
-      </c>
+          <t>霞发改审批〔2026〕94号</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>霞浦县总医院</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>霞浦县县域</t>
-        </is>
-      </c>
+          <t>霞浦县长春镇人民政府</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr"/>
       <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>申请超长期特别国债资金及地方财政配套</t>
-        </is>
-      </c>
+      <c r="H2" s="3" t="inlineStr"/>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482412.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202610/t20261016_2489801.htm</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>霞浦县沙江镇涵江村人居环境及生产道路提升项目</t>
+          <t>霞浦县松山农产品交易市场建设项目资金来源方式</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>可研批复</t>
+          <t>变更撤销类</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕79号</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>151.73</v>
-      </c>
+          <t>霞发改审批〔2026〕93号</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>霞浦县沙江镇人民政府</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>霞浦县沙江镇涵江村</t>
-        </is>
-      </c>
+          <t>霞浦县宾海融合投资发展有限公司</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>申请中央专项彩票公益金</t>
-        </is>
-      </c>
+      <c r="H3" s="3" t="inlineStr"/>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260901_2479035.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202610/t20261016_2489798.htm</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>霞浦县松港街道八斗浿村道路沿线设施及休闲文化广场改造提升项目</t>
+          <t>霞浦县县域医共体设备更新项目</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -2823,48 +2913,48 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕76号</t>
+          <t>霞发改审批〔2026〕84号</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>138.66</v>
+        <v>2789.32</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>霞浦县人民政府松港街道办事处</t>
+          <t>霞浦县总医院</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>霞浦县松港街道八斗浿村</t>
+          <t>霞浦县县域</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>申请中央专项彩票公益金</t>
+          <t>申请超长期特别国债资金及地方财政配套</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260901_2479026.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260916_2482412.htm</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>霞浦县松城街道青福村道路沿线设施提升及人居环境改造项目</t>
+          <t>霞浦县沙江镇涵江村人居环境及生产道路提升项目</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -2874,20 +2964,20 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕75号</t>
+          <t>霞发改审批〔2026〕79号</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>174.79</v>
+        <v>151.73</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>霞浦县人民政府松城街道办事处</t>
+          <t>霞浦县沙江镇人民政府</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>霞浦县松城街道青福村</t>
+          <t>霞浦县沙江镇涵江村</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
@@ -2898,122 +2988,142 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202608/t20260817_2476032.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260901_2479035.htm</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>霞浦县县域医共体资源共享项目</t>
+          <t>霞浦县松港街道八斗浿村道路沿线设施及休闲文化广场改造提升项目</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>变更撤销类</t>
+          <t>可研批复</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕73号</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr"/>
+          <t>霞发改审批〔2026〕76号</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>138.66</v>
+      </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>霞浦县总医院</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr"/>
+          <t>霞浦县人民政府松港街道办事处</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>霞浦县松港街道八斗浿村</t>
+        </is>
+      </c>
       <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>申请中央专项彩票公益金</t>
+        </is>
+      </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202608/t20260803_2473770.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202609/t20260901_2479026.htm</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>霞浦县公立医院能力提升项目</t>
+          <t>霞浦县松城街道青福村道路沿线设施提升及人居环境改造项目</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>变更撤销类</t>
+          <t>可研批复</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕72号</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr"/>
+          <t>霞发改审批〔2026〕75号</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>174.79</v>
+      </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>霞浦县总医院</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr"/>
+          <t>霞浦县人民政府松城街道办事处</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>霞浦县松城街道青福村</t>
+        </is>
+      </c>
       <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>申请中央专项彩票公益金</t>
+        </is>
+      </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202608/t20260803_2473766.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202608/t20260817_2476032.htm</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>霞浦县长春赤沙二级渔港</t>
+          <t>霞浦县县域医共体资源共享项目</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>可研批复</t>
+          <t>变更撤销类</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕71号</t>
+          <t>霞发改审批〔2026〕73号</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>霞浦县时代渔港建设有限公司</t>
+          <t>霞浦县总医院</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr"/>
@@ -3031,77 +3141,71 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202608/t20260803_2473764.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202608/t20260803_2473770.htm</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>霞浦县第六中学高中部迁建项目</t>
+          <t>霞浦县公立医院能力提升项目</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>可研批复</t>
+          <t>变更撤销类</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕61号</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>28247.16</v>
-      </c>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>霞浦县体育北路北侧、东利路西侧（六中新校初中部南侧）</t>
-        </is>
-      </c>
+          <t>霞发改审批〔2026〕72号</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>霞浦县总医院</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr"/>
       <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>申请上级政策性资金、县财政配套及业主自筹</t>
-        </is>
-      </c>
+      <c r="H9" s="3" t="inlineStr"/>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202607/t20260701_2467433.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202608/t20260803_2473766.htm</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>同意霞浦县三沙农渔产品交易中心及配套设施工程项目法人</t>
+          <t>霞浦县长春赤沙二级渔港</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>变更撤销类</t>
+          <t>可研批复</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕55号</t>
+          <t>霞发改审批〔2026〕71号</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>霞浦县三沙镇人民政府</t>
+          <t>霞浦县时代渔港建设有限公司</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr"/>
@@ -3109,24 +3213,24 @@
       <c r="H10" s="3" t="inlineStr"/>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202606/t20260615_2464195.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202608/t20260803_2473764.htm</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>福建省霞浦县北壁乡四门桥水闸除险加固工程</t>
+          <t>霞浦县第六中学高中部迁建项目</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -3136,48 +3240,44 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕48号</t>
+          <t>霞发改审批〔2026〕61号</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>2765.41</v>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>霞浦县北壁乡人民政府</t>
-        </is>
-      </c>
+        <v>28247.16</v>
+      </c>
+      <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>霞浦县北壁乡四门桥村</t>
+          <t>霞浦县体育北路北侧、东利路西侧（六中新校初中部南侧）</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr"/>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>中央预算内资金与县级财政配套</t>
+          <t>申请上级政策性资金、县财政配套及业主自筹</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459212.htm</t>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202607/t20260701_2467433.htm</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>同意霞浦县水门片区冷链物流项目法人</t>
+          <t>同意霞浦县三沙农渔产品交易中心及配套设施工程项目法人</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -3187,13 +3287,13 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>霞发改审批〔2026〕42号</t>
+          <t>霞发改审批〔2026〕55号</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>霞浦县水门畲族乡人民政府</t>
+          <t>霞浦县三沙镇人民政府</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr"/>
@@ -3201,15 +3301,107 @@
       <c r="H12" s="3" t="inlineStr"/>
       <c r="I12" s="3" t="inlineStr">
         <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202606/t20260615_2464195.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>福建省霞浦县北壁乡四门桥水闸除险加固工程</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>可研批复</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>霞发改审批〔2026〕48号</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>2765.41</v>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>霞浦县北壁乡人民政府</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>霞浦县北壁乡四门桥村</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>中央预算内资金与县级财政配套</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459212.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>同意霞浦县水门片区冷链物流项目法人</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>变更撤销类</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>霞发改审批〔2026〕42号</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>霞浦县水门畲族乡人民政府</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
           <t>2026-05-09</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="K14" s="3" t="inlineStr">
         <is>
           <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459204.htm</t>
         </is>

</xml_diff>

<commit_message>
auto: 产出更新 2026-10-31 13:22
</commit_message>
<xml_diff>
--- a/霞浦发改批复_近半年.xlsx
+++ b/霞浦发改批复_近半年.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2578,159 +2578,6 @@
       <c r="K41" s="3" t="inlineStr">
         <is>
           <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202605/t20260521_2459207.htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>福建省霞浦县海洋牧场深水抗风浪网箱养殖项目</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>可研批复</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>霞发改审批〔2026〕39号</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="n">
-        <v>24014</v>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t>福建省霞浦县光大渔港开发有限公司</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>霞浦县长春镇加竹村长草屿附近海域</t>
-        </is>
-      </c>
-      <c r="G42" s="3" t="inlineStr"/>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>申请专项债资金及财政资金</t>
-        </is>
-      </c>
-      <c r="I42" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="J42" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="K42" s="3" t="inlineStr">
-        <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202604/t20260430_2455988.htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>霞浦县松城街道西南片区老旧小区改造（四期）</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>设计批复</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>霞发改审批〔2026〕40号</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="n">
-        <v>5843.66</v>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>霞浦县人民政府松城街道办事处</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>霞浦县松城街道</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="inlineStr"/>
-      <c r="H43" s="3" t="inlineStr">
-        <is>
-          <t>申请专项债资金</t>
-        </is>
-      </c>
-      <c r="I43" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="J43" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="K43" s="3" t="inlineStr">
-        <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202604/t20260430_2455983.htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>福建省霞浦县海洋牧场深水抗风浪网箱养殖项目</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>设计批复</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>霞发改审批〔2026〕41号</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="n">
-        <v>23938.04</v>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>福建省霞浦县光大渔港开发有限公司</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>霞浦县长春镇加竹村长草屿附近海域</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr"/>
-      <c r="H44" s="3" t="inlineStr">
-        <is>
-          <t>申请专项债资金及财政资金</t>
-        </is>
-      </c>
-      <c r="I44" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="J44" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="K44" s="3" t="inlineStr">
-        <is>
-          <t>http://www.xiapu.gov.cn/zwgk/gkzl/bmzfxxgk/zfbm/xfzhggj/gkml/zdgkxx/202604/t20260430_2455979.htm</t>
         </is>
       </c>
     </row>

</xml_diff>